<commit_message>
Ajustes de planilha orçamentária
</commit_message>
<xml_diff>
--- a/banco_dados_orcamentario_onasp.xlsx
+++ b/banco_dados_orcamentario_onasp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://justicagovbr-my.sharepoint.com/personal/marcelo_cortez_mj_gov_br1/Documents/1. SENAPPEN/2. OUVIDORIA/GITHUB/FOMENTO-ONASP/FOMENTO-ONASP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{F20D0DE5-6B18-4F7F-97E9-7D6B0EAC69D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3859DD02-295D-45E7-9130-3B708331CC9E}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="13_ncr:1_{F20D0DE5-6B18-4F7F-97E9-7D6B0EAC69D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{846BEBBF-DBC9-407E-BC4C-67796F431E3E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="105">
   <si>
     <t>ID</t>
   </si>
@@ -310,6 +310,45 @@
   </si>
   <si>
     <t>Itens</t>
+  </si>
+  <si>
+    <t>Processo SEI</t>
+  </si>
+  <si>
+    <t>08016.004858/2026-23</t>
+  </si>
+  <si>
+    <t>Link do Processo SEI</t>
+  </si>
+  <si>
+    <t>https://sei.mj.gov.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=39457500</t>
+  </si>
+  <si>
+    <t>08016.009541/2026-83</t>
+  </si>
+  <si>
+    <t>https://sei.mj.gov.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=40118887</t>
+  </si>
+  <si>
+    <t>08016.003997/2026-30</t>
+  </si>
+  <si>
+    <t>https://sei.mj.gov.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=39355451</t>
+  </si>
+  <si>
+    <t>Em execução</t>
+  </si>
+  <si>
+    <t>Empenho</t>
+  </si>
+  <si>
+    <t>Link do Empenho</t>
+  </si>
+  <si>
+    <t>Ordem Bancária</t>
+  </si>
+  <si>
+    <t>Link Ordem Bancária</t>
   </si>
 </sst>
 </file>
@@ -319,7 +358,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\R\$\ #,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -344,6 +383,18 @@
     <font>
       <sz val="11"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F3763"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -521,10 +572,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -584,11 +636,124 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -704,20 +869,30 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tb_orcamento_onasp" displayName="tb_orcamento_onasp" ref="A1:K11">
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tb_orcamento_onasp" displayName="tb_orcamento_onasp" ref="A1:Q11">
+  <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Frente"/>
-    <tableColumn id="15" xr3:uid="{D914D5DF-272E-4DC3-A6F6-335470FE0AB3}" name="Itens" dataDxfId="1"/>
-    <tableColumn id="16" xr3:uid="{6A41EEBC-C904-4DFD-ADDC-3498EB40FBF3}" name="Natureza" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Modalidade" dataDxfId="2"/>
+    <tableColumn id="15" xr3:uid="{D914D5DF-272E-4DC3-A6F6-335470FE0AB3}" name="Itens" dataDxfId="8"/>
+    <tableColumn id="16" xr3:uid="{6A41EEBC-C904-4DFD-ADDC-3498EB40FBF3}" name="Natureza" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Modalidade" dataDxfId="6"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="UFs/Abrangência"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Quantidade"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Unidade"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Valor Total (R$)"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Valor Unitário (R$)"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Status"/>
+    <tableColumn id="3" xr3:uid="{88B19836-1B82-4EF8-8262-E6176FE711DE}" name="Processo SEI" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{552AA666-E583-4D36-947C-13CD935F3A75}" name="Link do Processo SEI" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{3D181ED2-691D-47A7-B38A-6479B9541618}" name="Empenho" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{47679C53-0F0B-4B30-B86B-2CFDE3582706}" name="Link do Empenho" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{C311DB84-7F79-49B7-ACA8-9BBD21A0B19E}" name="Ordem Bancária" dataDxfId="1"/>
+    <tableColumn id="18" xr3:uid="{F6EDDDF3-6451-4044-8993-8EB708FE90CB}" name="Link Ordem Bancária" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -872,20 +1047,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W117"/>
+  <dimension ref="A1:V117"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" customWidth="1"/>
-    <col min="2" max="4" width="37.88671875" customWidth="1"/>
-    <col min="5" max="5" width="16.44140625" customWidth="1"/>
-    <col min="6" max="6" width="37.88671875" customWidth="1"/>
+    <col min="2" max="3" width="37.88671875" customWidth="1"/>
+    <col min="4" max="4" width="37.88671875" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="16.44140625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="37.88671875" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="12.109375" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="10" width="18.5546875" customWidth="1"/>
     <col min="11" max="11" width="13.5546875" customWidth="1"/>
+    <col min="12" max="12" width="22.5546875" customWidth="1"/>
+    <col min="13" max="13" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -919,20 +1101,31 @@
       <c r="K1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
+      <c r="L1" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="P1" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q1" s="23" t="s">
+        <v>104</v>
+      </c>
       <c r="R1" s="20"/>
       <c r="S1" s="20"/>
       <c r="T1" s="20"/>
       <c r="U1" s="20"/>
       <c r="V1" s="20"/>
-      <c r="W1" s="20"/>
-    </row>
-    <row r="2" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>14</v>
       </c>
@@ -965,10 +1158,14 @@
         <v>212500</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
+        <v>100</v>
+      </c>
+      <c r="L2" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="M2" s="21" t="s">
+        <v>95</v>
+      </c>
       <c r="N2" s="20"/>
       <c r="O2" s="20"/>
       <c r="P2" s="20"/>
@@ -978,9 +1175,8 @@
       <c r="T2" s="20"/>
       <c r="U2" s="20"/>
       <c r="V2" s="20"/>
-      <c r="W2" s="20"/>
-    </row>
-    <row r="3" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
@@ -1013,10 +1209,14 @@
         <v>2407.4074074074074</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
+        <v>100</v>
+      </c>
+      <c r="L3" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="M3" s="21" t="s">
+        <v>99</v>
+      </c>
       <c r="N3" s="20"/>
       <c r="O3" s="20"/>
       <c r="P3" s="20"/>
@@ -1026,9 +1226,8 @@
       <c r="T3" s="20"/>
       <c r="U3" s="20"/>
       <c r="V3" s="20"/>
-      <c r="W3" s="20"/>
-    </row>
-    <row r="4" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>23</v>
       </c>
@@ -1061,10 +1260,14 @@
         <v>2777.7777777777778</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
+        <v>100</v>
+      </c>
+      <c r="L4" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>99</v>
+      </c>
       <c r="N4" s="20"/>
       <c r="O4" s="20"/>
       <c r="P4" s="20"/>
@@ -1074,9 +1277,8 @@
       <c r="T4" s="20"/>
       <c r="U4" s="20"/>
       <c r="V4" s="20"/>
-      <c r="W4" s="20"/>
-    </row>
-    <row r="5" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>25</v>
       </c>
@@ -1109,10 +1311,14 @@
         <v>5000</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
+        <v>100</v>
+      </c>
+      <c r="L5" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="M5" s="21" t="s">
+        <v>99</v>
+      </c>
       <c r="N5" s="20"/>
       <c r="O5" s="20"/>
       <c r="P5" s="20"/>
@@ -1122,9 +1328,8 @@
       <c r="T5" s="20"/>
       <c r="U5" s="20"/>
       <c r="V5" s="20"/>
-      <c r="W5" s="20"/>
-    </row>
-    <row r="6" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>27</v>
       </c>
@@ -1157,10 +1362,14 @@
         <v>18129.166666666668</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
+        <v>100</v>
+      </c>
+      <c r="L6" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="M6" s="21" t="s">
+        <v>97</v>
+      </c>
       <c r="N6" s="20"/>
       <c r="O6" s="20"/>
       <c r="P6" s="20"/>
@@ -1170,9 +1379,8 @@
       <c r="T6" s="20"/>
       <c r="U6" s="20"/>
       <c r="V6" s="20"/>
-      <c r="W6" s="20"/>
-    </row>
-    <row r="7" spans="1:23" ht="27.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:22" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>29</v>
       </c>
@@ -1208,7 +1416,7 @@
         <v>20</v>
       </c>
       <c r="L7" s="20"/>
-      <c r="M7" s="20"/>
+      <c r="M7" s="22"/>
       <c r="N7" s="20"/>
       <c r="O7" s="20"/>
       <c r="P7" s="20"/>
@@ -1218,9 +1426,8 @@
       <c r="T7" s="20"/>
       <c r="U7" s="20"/>
       <c r="V7" s="20"/>
-      <c r="W7" s="20"/>
-    </row>
-    <row r="8" spans="1:23" ht="27.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:22" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>33</v>
       </c>
@@ -1256,7 +1463,7 @@
         <v>20</v>
       </c>
       <c r="L8" s="20"/>
-      <c r="M8" s="20"/>
+      <c r="M8" s="22"/>
       <c r="N8" s="20"/>
       <c r="O8" s="20"/>
       <c r="P8" s="20"/>
@@ -1266,9 +1473,8 @@
       <c r="T8" s="20"/>
       <c r="U8" s="20"/>
       <c r="V8" s="20"/>
-      <c r="W8" s="20"/>
-    </row>
-    <row r="9" spans="1:23" ht="27.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:22" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>39</v>
       </c>
@@ -1304,7 +1510,7 @@
         <v>20</v>
       </c>
       <c r="L9" s="20"/>
-      <c r="M9" s="20"/>
+      <c r="M9" s="22"/>
       <c r="N9" s="20"/>
       <c r="O9" s="20"/>
       <c r="P9" s="20"/>
@@ -1314,9 +1520,8 @@
       <c r="T9" s="20"/>
       <c r="U9" s="20"/>
       <c r="V9" s="20"/>
-      <c r="W9" s="20"/>
-    </row>
-    <row r="10" spans="1:23" ht="27.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:22" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>44</v>
       </c>
@@ -1352,7 +1557,7 @@
         <v>20</v>
       </c>
       <c r="L10" s="20"/>
-      <c r="M10" s="20"/>
+      <c r="M10" s="22"/>
       <c r="N10" s="20"/>
       <c r="O10" s="20"/>
       <c r="P10" s="20"/>
@@ -1362,9 +1567,8 @@
       <c r="T10" s="20"/>
       <c r="U10" s="20"/>
       <c r="V10" s="20"/>
-      <c r="W10" s="20"/>
-    </row>
-    <row r="11" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>48</v>
       </c>
@@ -1398,7 +1602,7 @@
         <v>20</v>
       </c>
       <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
+      <c r="M11" s="22"/>
       <c r="N11" s="20"/>
       <c r="O11" s="20"/>
       <c r="P11" s="20"/>
@@ -1408,9 +1612,8 @@
       <c r="T11" s="20"/>
       <c r="U11" s="20"/>
       <c r="V11" s="20"/>
-      <c r="W11" s="20"/>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="20"/>
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
@@ -1433,9 +1636,8 @@
       <c r="T12" s="20"/>
       <c r="U12" s="20"/>
       <c r="V12" s="20"/>
-      <c r="W12" s="20"/>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="20"/>
       <c r="B13" s="20"/>
       <c r="C13" s="20"/>
@@ -1458,9 +1660,8 @@
       <c r="T13" s="20"/>
       <c r="U13" s="20"/>
       <c r="V13" s="20"/>
-      <c r="W13" s="20"/>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="20"/>
       <c r="B14" s="20"/>
       <c r="C14" s="20"/>
@@ -1483,9 +1684,8 @@
       <c r="T14" s="20"/>
       <c r="U14" s="20"/>
       <c r="V14" s="20"/>
-      <c r="W14" s="20"/>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="20"/>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -1508,9 +1708,8 @@
       <c r="T15" s="20"/>
       <c r="U15" s="20"/>
       <c r="V15" s="20"/>
-      <c r="W15" s="20"/>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="20"/>
       <c r="B16" s="20"/>
       <c r="C16" s="20"/>
@@ -1533,9 +1732,8 @@
       <c r="T16" s="20"/>
       <c r="U16" s="20"/>
       <c r="V16" s="20"/>
-      <c r="W16" s="20"/>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" s="20"/>
       <c r="B17" s="20"/>
       <c r="C17" s="20"/>
@@ -1558,9 +1756,8 @@
       <c r="T17" s="20"/>
       <c r="U17" s="20"/>
       <c r="V17" s="20"/>
-      <c r="W17" s="20"/>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" s="20"/>
       <c r="B18" s="20"/>
       <c r="C18" s="20"/>
@@ -1583,9 +1780,8 @@
       <c r="T18" s="20"/>
       <c r="U18" s="20"/>
       <c r="V18" s="20"/>
-      <c r="W18" s="20"/>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19" s="20"/>
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
@@ -1608,9 +1804,8 @@
       <c r="T19" s="20"/>
       <c r="U19" s="20"/>
       <c r="V19" s="20"/>
-      <c r="W19" s="20"/>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="20"/>
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
@@ -1633,9 +1828,8 @@
       <c r="T20" s="20"/>
       <c r="U20" s="20"/>
       <c r="V20" s="20"/>
-      <c r="W20" s="20"/>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21" s="20"/>
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
@@ -1658,9 +1852,8 @@
       <c r="T21" s="20"/>
       <c r="U21" s="20"/>
       <c r="V21" s="20"/>
-      <c r="W21" s="20"/>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" s="20"/>
       <c r="B22" s="20"/>
       <c r="C22" s="20"/>
@@ -1683,9 +1876,8 @@
       <c r="T22" s="20"/>
       <c r="U22" s="20"/>
       <c r="V22" s="20"/>
-      <c r="W22" s="20"/>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23" s="20"/>
       <c r="B23" s="20"/>
       <c r="C23" s="20"/>
@@ -1708,9 +1900,8 @@
       <c r="T23" s="20"/>
       <c r="U23" s="20"/>
       <c r="V23" s="20"/>
-      <c r="W23" s="20"/>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24" s="20"/>
       <c r="B24" s="20"/>
       <c r="C24" s="20"/>
@@ -1733,9 +1924,8 @@
       <c r="T24" s="20"/>
       <c r="U24" s="20"/>
       <c r="V24" s="20"/>
-      <c r="W24" s="20"/>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25" s="20"/>
       <c r="B25" s="20"/>
       <c r="C25" s="20"/>
@@ -1758,9 +1948,8 @@
       <c r="T25" s="20"/>
       <c r="U25" s="20"/>
       <c r="V25" s="20"/>
-      <c r="W25" s="20"/>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" s="20"/>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
@@ -1783,9 +1972,8 @@
       <c r="T26" s="20"/>
       <c r="U26" s="20"/>
       <c r="V26" s="20"/>
-      <c r="W26" s="20"/>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" s="20"/>
       <c r="B27" s="20"/>
       <c r="C27" s="20"/>
@@ -1808,9 +1996,8 @@
       <c r="T27" s="20"/>
       <c r="U27" s="20"/>
       <c r="V27" s="20"/>
-      <c r="W27" s="20"/>
-    </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" s="20"/>
       <c r="B28" s="20"/>
       <c r="C28" s="20"/>
@@ -1833,9 +2020,8 @@
       <c r="T28" s="20"/>
       <c r="U28" s="20"/>
       <c r="V28" s="20"/>
-      <c r="W28" s="20"/>
-    </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A29" s="20"/>
       <c r="B29" s="20"/>
       <c r="C29" s="20"/>
@@ -1858,9 +2044,8 @@
       <c r="T29" s="20"/>
       <c r="U29" s="20"/>
       <c r="V29" s="20"/>
-      <c r="W29" s="20"/>
-    </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A30" s="20"/>
       <c r="B30" s="20"/>
       <c r="C30" s="20"/>
@@ -1883,9 +2068,8 @@
       <c r="T30" s="20"/>
       <c r="U30" s="20"/>
       <c r="V30" s="20"/>
-      <c r="W30" s="20"/>
-    </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A31" s="20"/>
       <c r="B31" s="20"/>
       <c r="C31" s="20"/>
@@ -1908,9 +2092,8 @@
       <c r="T31" s="20"/>
       <c r="U31" s="20"/>
       <c r="V31" s="20"/>
-      <c r="W31" s="20"/>
-    </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A32" s="20"/>
       <c r="B32" s="20"/>
       <c r="C32" s="20"/>
@@ -1933,9 +2116,8 @@
       <c r="T32" s="20"/>
       <c r="U32" s="20"/>
       <c r="V32" s="20"/>
-      <c r="W32" s="20"/>
-    </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A33" s="20"/>
       <c r="B33" s="20"/>
       <c r="C33" s="20"/>
@@ -1958,9 +2140,8 @@
       <c r="T33" s="20"/>
       <c r="U33" s="20"/>
       <c r="V33" s="20"/>
-      <c r="W33" s="20"/>
-    </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A34" s="20"/>
       <c r="B34" s="20"/>
       <c r="C34" s="20"/>
@@ -1983,9 +2164,8 @@
       <c r="T34" s="20"/>
       <c r="U34" s="20"/>
       <c r="V34" s="20"/>
-      <c r="W34" s="20"/>
-    </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A35" s="20"/>
       <c r="B35" s="20"/>
       <c r="C35" s="20"/>
@@ -2008,9 +2188,8 @@
       <c r="T35" s="20"/>
       <c r="U35" s="20"/>
       <c r="V35" s="20"/>
-      <c r="W35" s="20"/>
-    </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A36" s="20"/>
       <c r="B36" s="20"/>
       <c r="C36" s="20"/>
@@ -2033,9 +2212,8 @@
       <c r="T36" s="20"/>
       <c r="U36" s="20"/>
       <c r="V36" s="20"/>
-      <c r="W36" s="20"/>
-    </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A37" s="20"/>
       <c r="B37" s="20"/>
       <c r="C37" s="20"/>
@@ -2058,9 +2236,8 @@
       <c r="T37" s="20"/>
       <c r="U37" s="20"/>
       <c r="V37" s="20"/>
-      <c r="W37" s="20"/>
-    </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A38" s="20"/>
       <c r="B38" s="20"/>
       <c r="C38" s="20"/>
@@ -2083,9 +2260,8 @@
       <c r="T38" s="20"/>
       <c r="U38" s="20"/>
       <c r="V38" s="20"/>
-      <c r="W38" s="20"/>
-    </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" s="20"/>
       <c r="B39" s="20"/>
       <c r="C39" s="20"/>
@@ -2108,9 +2284,8 @@
       <c r="T39" s="20"/>
       <c r="U39" s="20"/>
       <c r="V39" s="20"/>
-      <c r="W39" s="20"/>
-    </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A40" s="20"/>
       <c r="B40" s="20"/>
       <c r="C40" s="20"/>
@@ -2133,9 +2308,8 @@
       <c r="T40" s="20"/>
       <c r="U40" s="20"/>
       <c r="V40" s="20"/>
-      <c r="W40" s="20"/>
-    </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A41" s="20"/>
       <c r="B41" s="20"/>
       <c r="C41" s="20"/>
@@ -2158,9 +2332,8 @@
       <c r="T41" s="20"/>
       <c r="U41" s="20"/>
       <c r="V41" s="20"/>
-      <c r="W41" s="20"/>
-    </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A42" s="20"/>
       <c r="B42" s="20"/>
       <c r="C42" s="20"/>
@@ -2183,9 +2356,8 @@
       <c r="T42" s="20"/>
       <c r="U42" s="20"/>
       <c r="V42" s="20"/>
-      <c r="W42" s="20"/>
-    </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A43" s="20"/>
       <c r="B43" s="20"/>
       <c r="C43" s="20"/>
@@ -2208,9 +2380,8 @@
       <c r="T43" s="20"/>
       <c r="U43" s="20"/>
       <c r="V43" s="20"/>
-      <c r="W43" s="20"/>
-    </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A44" s="20"/>
       <c r="B44" s="20"/>
       <c r="C44" s="20"/>
@@ -2233,9 +2404,8 @@
       <c r="T44" s="20"/>
       <c r="U44" s="20"/>
       <c r="V44" s="20"/>
-      <c r="W44" s="20"/>
-    </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A45" s="20"/>
       <c r="B45" s="20"/>
       <c r="C45" s="20"/>
@@ -2258,9 +2428,8 @@
       <c r="T45" s="20"/>
       <c r="U45" s="20"/>
       <c r="V45" s="20"/>
-      <c r="W45" s="20"/>
-    </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A46" s="20"/>
       <c r="B46" s="20"/>
       <c r="C46" s="20"/>
@@ -2283,9 +2452,8 @@
       <c r="T46" s="20"/>
       <c r="U46" s="20"/>
       <c r="V46" s="20"/>
-      <c r="W46" s="20"/>
-    </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
@@ -2308,9 +2476,8 @@
       <c r="T47" s="20"/>
       <c r="U47" s="20"/>
       <c r="V47" s="20"/>
-      <c r="W47" s="20"/>
-    </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
       <c r="C48" s="20"/>
@@ -2333,9 +2500,8 @@
       <c r="T48" s="20"/>
       <c r="U48" s="20"/>
       <c r="V48" s="20"/>
-      <c r="W48" s="20"/>
-    </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="20"/>
@@ -2358,9 +2524,8 @@
       <c r="T49" s="20"/>
       <c r="U49" s="20"/>
       <c r="V49" s="20"/>
-      <c r="W49" s="20"/>
-    </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A50" s="20"/>
       <c r="B50" s="20"/>
       <c r="C50" s="20"/>
@@ -2383,9 +2548,8 @@
       <c r="T50" s="20"/>
       <c r="U50" s="20"/>
       <c r="V50" s="20"/>
-      <c r="W50" s="20"/>
-    </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="20"/>
@@ -2408,9 +2572,8 @@
       <c r="T51" s="20"/>
       <c r="U51" s="20"/>
       <c r="V51" s="20"/>
-      <c r="W51" s="20"/>
-    </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A52" s="20"/>
       <c r="B52" s="20"/>
       <c r="C52" s="20"/>
@@ -2433,9 +2596,8 @@
       <c r="T52" s="20"/>
       <c r="U52" s="20"/>
       <c r="V52" s="20"/>
-      <c r="W52" s="20"/>
-    </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A53" s="20"/>
       <c r="B53" s="20"/>
       <c r="C53" s="20"/>
@@ -2458,9 +2620,8 @@
       <c r="T53" s="20"/>
       <c r="U53" s="20"/>
       <c r="V53" s="20"/>
-      <c r="W53" s="20"/>
-    </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A54" s="20"/>
       <c r="B54" s="20"/>
       <c r="C54" s="20"/>
@@ -2483,9 +2644,8 @@
       <c r="T54" s="20"/>
       <c r="U54" s="20"/>
       <c r="V54" s="20"/>
-      <c r="W54" s="20"/>
-    </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A55" s="20"/>
       <c r="B55" s="20"/>
       <c r="C55" s="20"/>
@@ -2508,9 +2668,8 @@
       <c r="T55" s="20"/>
       <c r="U55" s="20"/>
       <c r="V55" s="20"/>
-      <c r="W55" s="20"/>
-    </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A56" s="20"/>
       <c r="B56" s="20"/>
       <c r="C56" s="20"/>
@@ -2533,9 +2692,8 @@
       <c r="T56" s="20"/>
       <c r="U56" s="20"/>
       <c r="V56" s="20"/>
-      <c r="W56" s="20"/>
-    </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A57" s="20"/>
       <c r="B57" s="20"/>
       <c r="C57" s="20"/>
@@ -2558,9 +2716,8 @@
       <c r="T57" s="20"/>
       <c r="U57" s="20"/>
       <c r="V57" s="20"/>
-      <c r="W57" s="20"/>
-    </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A58" s="20"/>
       <c r="B58" s="20"/>
       <c r="C58" s="20"/>
@@ -2583,9 +2740,8 @@
       <c r="T58" s="20"/>
       <c r="U58" s="20"/>
       <c r="V58" s="20"/>
-      <c r="W58" s="20"/>
-    </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A59" s="20"/>
       <c r="B59" s="20"/>
       <c r="C59" s="20"/>
@@ -2608,9 +2764,8 @@
       <c r="T59" s="20"/>
       <c r="U59" s="20"/>
       <c r="V59" s="20"/>
-      <c r="W59" s="20"/>
-    </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A60" s="20"/>
       <c r="B60" s="20"/>
       <c r="C60" s="20"/>
@@ -2633,9 +2788,8 @@
       <c r="T60" s="20"/>
       <c r="U60" s="20"/>
       <c r="V60" s="20"/>
-      <c r="W60" s="20"/>
-    </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A61" s="20"/>
       <c r="B61" s="20"/>
       <c r="C61" s="20"/>
@@ -2658,9 +2812,8 @@
       <c r="T61" s="20"/>
       <c r="U61" s="20"/>
       <c r="V61" s="20"/>
-      <c r="W61" s="20"/>
-    </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A62" s="20"/>
       <c r="B62" s="20"/>
       <c r="C62" s="20"/>
@@ -2683,9 +2836,8 @@
       <c r="T62" s="20"/>
       <c r="U62" s="20"/>
       <c r="V62" s="20"/>
-      <c r="W62" s="20"/>
-    </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A63" s="20"/>
       <c r="B63" s="20"/>
       <c r="C63" s="20"/>
@@ -2708,9 +2860,8 @@
       <c r="T63" s="20"/>
       <c r="U63" s="20"/>
       <c r="V63" s="20"/>
-      <c r="W63" s="20"/>
-    </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A64" s="20"/>
       <c r="B64" s="20"/>
       <c r="C64" s="20"/>
@@ -2733,9 +2884,8 @@
       <c r="T64" s="20"/>
       <c r="U64" s="20"/>
       <c r="V64" s="20"/>
-      <c r="W64" s="20"/>
-    </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="65" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A65" s="20"/>
       <c r="B65" s="20"/>
       <c r="C65" s="20"/>
@@ -2758,9 +2908,8 @@
       <c r="T65" s="20"/>
       <c r="U65" s="20"/>
       <c r="V65" s="20"/>
-      <c r="W65" s="20"/>
-    </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="66" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A66" s="20"/>
       <c r="B66" s="20"/>
       <c r="C66" s="20"/>
@@ -2783,9 +2932,8 @@
       <c r="T66" s="20"/>
       <c r="U66" s="20"/>
       <c r="V66" s="20"/>
-      <c r="W66" s="20"/>
-    </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="67" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A67" s="20"/>
       <c r="B67" s="20"/>
       <c r="C67" s="20"/>
@@ -2808,9 +2956,8 @@
       <c r="T67" s="20"/>
       <c r="U67" s="20"/>
       <c r="V67" s="20"/>
-      <c r="W67" s="20"/>
-    </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="68" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A68" s="20"/>
       <c r="B68" s="20"/>
       <c r="C68" s="20"/>
@@ -2833,9 +2980,8 @@
       <c r="T68" s="20"/>
       <c r="U68" s="20"/>
       <c r="V68" s="20"/>
-      <c r="W68" s="20"/>
-    </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="69" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A69" s="20"/>
       <c r="B69" s="20"/>
       <c r="C69" s="20"/>
@@ -2858,9 +3004,8 @@
       <c r="T69" s="20"/>
       <c r="U69" s="20"/>
       <c r="V69" s="20"/>
-      <c r="W69" s="20"/>
-    </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A70" s="20"/>
       <c r="B70" s="20"/>
       <c r="C70" s="20"/>
@@ -2883,9 +3028,8 @@
       <c r="T70" s="20"/>
       <c r="U70" s="20"/>
       <c r="V70" s="20"/>
-      <c r="W70" s="20"/>
-    </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A71" s="20"/>
       <c r="B71" s="20"/>
       <c r="C71" s="20"/>
@@ -2908,9 +3052,8 @@
       <c r="T71" s="20"/>
       <c r="U71" s="20"/>
       <c r="V71" s="20"/>
-      <c r="W71" s="20"/>
-    </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="72" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A72" s="20"/>
       <c r="B72" s="20"/>
       <c r="C72" s="20"/>
@@ -2933,9 +3076,8 @@
       <c r="T72" s="20"/>
       <c r="U72" s="20"/>
       <c r="V72" s="20"/>
-      <c r="W72" s="20"/>
-    </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="73" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A73" s="20"/>
       <c r="B73" s="20"/>
       <c r="C73" s="20"/>
@@ -2958,9 +3100,8 @@
       <c r="T73" s="20"/>
       <c r="U73" s="20"/>
       <c r="V73" s="20"/>
-      <c r="W73" s="20"/>
-    </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A74" s="20"/>
       <c r="B74" s="20"/>
       <c r="C74" s="20"/>
@@ -2983,9 +3124,8 @@
       <c r="T74" s="20"/>
       <c r="U74" s="20"/>
       <c r="V74" s="20"/>
-      <c r="W74" s="20"/>
-    </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="75" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A75" s="20"/>
       <c r="B75" s="20"/>
       <c r="C75" s="20"/>
@@ -3008,9 +3148,8 @@
       <c r="T75" s="20"/>
       <c r="U75" s="20"/>
       <c r="V75" s="20"/>
-      <c r="W75" s="20"/>
-    </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="76" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A76" s="20"/>
       <c r="B76" s="20"/>
       <c r="C76" s="20"/>
@@ -3033,9 +3172,8 @@
       <c r="T76" s="20"/>
       <c r="U76" s="20"/>
       <c r="V76" s="20"/>
-      <c r="W76" s="20"/>
-    </row>
-    <row r="77" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="77" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A77" s="20"/>
       <c r="B77" s="20"/>
       <c r="C77" s="20"/>
@@ -3058,9 +3196,8 @@
       <c r="T77" s="20"/>
       <c r="U77" s="20"/>
       <c r="V77" s="20"/>
-      <c r="W77" s="20"/>
-    </row>
-    <row r="78" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="78" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A78" s="20"/>
       <c r="B78" s="20"/>
       <c r="C78" s="20"/>
@@ -3083,9 +3220,8 @@
       <c r="T78" s="20"/>
       <c r="U78" s="20"/>
       <c r="V78" s="20"/>
-      <c r="W78" s="20"/>
-    </row>
-    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="79" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A79" s="20"/>
       <c r="B79" s="20"/>
       <c r="C79" s="20"/>
@@ -3108,9 +3244,8 @@
       <c r="T79" s="20"/>
       <c r="U79" s="20"/>
       <c r="V79" s="20"/>
-      <c r="W79" s="20"/>
-    </row>
-    <row r="80" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="80" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A80" s="20"/>
       <c r="B80" s="20"/>
       <c r="C80" s="20"/>
@@ -3133,9 +3268,8 @@
       <c r="T80" s="20"/>
       <c r="U80" s="20"/>
       <c r="V80" s="20"/>
-      <c r="W80" s="20"/>
-    </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="81" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A81" s="20"/>
       <c r="B81" s="20"/>
       <c r="C81" s="20"/>
@@ -3158,9 +3292,8 @@
       <c r="T81" s="20"/>
       <c r="U81" s="20"/>
       <c r="V81" s="20"/>
-      <c r="W81" s="20"/>
-    </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="82" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A82" s="20"/>
       <c r="B82" s="20"/>
       <c r="C82" s="20"/>
@@ -3183,9 +3316,8 @@
       <c r="T82" s="20"/>
       <c r="U82" s="20"/>
       <c r="V82" s="20"/>
-      <c r="W82" s="20"/>
-    </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83" s="20"/>
       <c r="B83" s="20"/>
       <c r="C83" s="20"/>
@@ -3208,9 +3340,8 @@
       <c r="T83" s="20"/>
       <c r="U83" s="20"/>
       <c r="V83" s="20"/>
-      <c r="W83" s="20"/>
-    </row>
-    <row r="84" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84" s="20"/>
       <c r="B84" s="20"/>
       <c r="C84" s="20"/>
@@ -3233,9 +3364,8 @@
       <c r="T84" s="20"/>
       <c r="U84" s="20"/>
       <c r="V84" s="20"/>
-      <c r="W84" s="20"/>
-    </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="85" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A85" s="20"/>
       <c r="B85" s="20"/>
       <c r="C85" s="20"/>
@@ -3258,9 +3388,8 @@
       <c r="T85" s="20"/>
       <c r="U85" s="20"/>
       <c r="V85" s="20"/>
-      <c r="W85" s="20"/>
-    </row>
-    <row r="86" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86" s="20"/>
       <c r="B86" s="20"/>
       <c r="C86" s="20"/>
@@ -3283,9 +3412,8 @@
       <c r="T86" s="20"/>
       <c r="U86" s="20"/>
       <c r="V86" s="20"/>
-      <c r="W86" s="20"/>
-    </row>
-    <row r="87" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="87" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A87" s="20"/>
       <c r="B87" s="20"/>
       <c r="C87" s="20"/>
@@ -3308,9 +3436,8 @@
       <c r="T87" s="20"/>
       <c r="U87" s="20"/>
       <c r="V87" s="20"/>
-      <c r="W87" s="20"/>
-    </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A88" s="20"/>
       <c r="B88" s="20"/>
       <c r="C88" s="20"/>
@@ -3333,9 +3460,8 @@
       <c r="T88" s="20"/>
       <c r="U88" s="20"/>
       <c r="V88" s="20"/>
-      <c r="W88" s="20"/>
-    </row>
-    <row r="89" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89" s="20"/>
       <c r="B89" s="20"/>
       <c r="C89" s="20"/>
@@ -3358,9 +3484,8 @@
       <c r="T89" s="20"/>
       <c r="U89" s="20"/>
       <c r="V89" s="20"/>
-      <c r="W89" s="20"/>
-    </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="90" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A90" s="20"/>
       <c r="B90" s="20"/>
       <c r="C90" s="20"/>
@@ -3383,9 +3508,8 @@
       <c r="T90" s="20"/>
       <c r="U90" s="20"/>
       <c r="V90" s="20"/>
-      <c r="W90" s="20"/>
-    </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="91" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A91" s="20"/>
       <c r="B91" s="20"/>
       <c r="C91" s="20"/>
@@ -3408,9 +3532,8 @@
       <c r="T91" s="20"/>
       <c r="U91" s="20"/>
       <c r="V91" s="20"/>
-      <c r="W91" s="20"/>
-    </row>
-    <row r="92" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="92" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A92" s="20"/>
       <c r="B92" s="20"/>
       <c r="C92" s="20"/>
@@ -3433,9 +3556,8 @@
       <c r="T92" s="20"/>
       <c r="U92" s="20"/>
       <c r="V92" s="20"/>
-      <c r="W92" s="20"/>
-    </row>
-    <row r="93" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="93" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A93" s="20"/>
       <c r="B93" s="20"/>
       <c r="C93" s="20"/>
@@ -3458,9 +3580,8 @@
       <c r="T93" s="20"/>
       <c r="U93" s="20"/>
       <c r="V93" s="20"/>
-      <c r="W93" s="20"/>
-    </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94" s="20"/>
       <c r="B94" s="20"/>
       <c r="C94" s="20"/>
@@ -3483,9 +3604,8 @@
       <c r="T94" s="20"/>
       <c r="U94" s="20"/>
       <c r="V94" s="20"/>
-      <c r="W94" s="20"/>
-    </row>
-    <row r="95" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="95" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A95" s="20"/>
       <c r="B95" s="20"/>
       <c r="C95" s="20"/>
@@ -3508,9 +3628,8 @@
       <c r="T95" s="20"/>
       <c r="U95" s="20"/>
       <c r="V95" s="20"/>
-      <c r="W95" s="20"/>
-    </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="96" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A96" s="20"/>
       <c r="B96" s="20"/>
       <c r="C96" s="20"/>
@@ -3533,9 +3652,8 @@
       <c r="T96" s="20"/>
       <c r="U96" s="20"/>
       <c r="V96" s="20"/>
-      <c r="W96" s="20"/>
-    </row>
-    <row r="97" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="97" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A97" s="20"/>
       <c r="B97" s="20"/>
       <c r="C97" s="20"/>
@@ -3558,9 +3676,8 @@
       <c r="T97" s="20"/>
       <c r="U97" s="20"/>
       <c r="V97" s="20"/>
-      <c r="W97" s="20"/>
-    </row>
-    <row r="98" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="98" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A98" s="20"/>
       <c r="B98" s="20"/>
       <c r="C98" s="20"/>
@@ -3583,9 +3700,8 @@
       <c r="T98" s="20"/>
       <c r="U98" s="20"/>
       <c r="V98" s="20"/>
-      <c r="W98" s="20"/>
-    </row>
-    <row r="99" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="99" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A99" s="20"/>
       <c r="B99" s="20"/>
       <c r="C99" s="20"/>
@@ -3608,9 +3724,8 @@
       <c r="T99" s="20"/>
       <c r="U99" s="20"/>
       <c r="V99" s="20"/>
-      <c r="W99" s="20"/>
-    </row>
-    <row r="100" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="100" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A100" s="20"/>
       <c r="B100" s="20"/>
       <c r="C100" s="20"/>
@@ -3633,9 +3748,8 @@
       <c r="T100" s="20"/>
       <c r="U100" s="20"/>
       <c r="V100" s="20"/>
-      <c r="W100" s="20"/>
-    </row>
-    <row r="101" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="101" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A101" s="20"/>
       <c r="B101" s="20"/>
       <c r="C101" s="20"/>
@@ -3658,9 +3772,8 @@
       <c r="T101" s="20"/>
       <c r="U101" s="20"/>
       <c r="V101" s="20"/>
-      <c r="W101" s="20"/>
-    </row>
-    <row r="102" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="102" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A102" s="20"/>
       <c r="B102" s="20"/>
       <c r="C102" s="20"/>
@@ -3683,9 +3796,8 @@
       <c r="T102" s="20"/>
       <c r="U102" s="20"/>
       <c r="V102" s="20"/>
-      <c r="W102" s="20"/>
-    </row>
-    <row r="103" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="103" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A103" s="20"/>
       <c r="B103" s="20"/>
       <c r="C103" s="20"/>
@@ -3708,9 +3820,8 @@
       <c r="T103" s="20"/>
       <c r="U103" s="20"/>
       <c r="V103" s="20"/>
-      <c r="W103" s="20"/>
-    </row>
-    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="104" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A104" s="20"/>
       <c r="B104" s="20"/>
       <c r="C104" s="20"/>
@@ -3733,9 +3844,8 @@
       <c r="T104" s="20"/>
       <c r="U104" s="20"/>
       <c r="V104" s="20"/>
-      <c r="W104" s="20"/>
-    </row>
-    <row r="105" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="105" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A105" s="20"/>
       <c r="B105" s="20"/>
       <c r="C105" s="20"/>
@@ -3758,9 +3868,8 @@
       <c r="T105" s="20"/>
       <c r="U105" s="20"/>
       <c r="V105" s="20"/>
-      <c r="W105" s="20"/>
-    </row>
-    <row r="106" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="106" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A106" s="20"/>
       <c r="B106" s="20"/>
       <c r="C106" s="20"/>
@@ -3783,9 +3892,8 @@
       <c r="T106" s="20"/>
       <c r="U106" s="20"/>
       <c r="V106" s="20"/>
-      <c r="W106" s="20"/>
-    </row>
-    <row r="107" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="107" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A107" s="20"/>
       <c r="B107" s="20"/>
       <c r="C107" s="20"/>
@@ -3808,9 +3916,8 @@
       <c r="T107" s="20"/>
       <c r="U107" s="20"/>
       <c r="V107" s="20"/>
-      <c r="W107" s="20"/>
-    </row>
-    <row r="108" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="108" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A108" s="20"/>
       <c r="B108" s="20"/>
       <c r="C108" s="20"/>
@@ -3833,9 +3940,8 @@
       <c r="T108" s="20"/>
       <c r="U108" s="20"/>
       <c r="V108" s="20"/>
-      <c r="W108" s="20"/>
-    </row>
-    <row r="109" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="109" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A109" s="20"/>
       <c r="B109" s="20"/>
       <c r="C109" s="20"/>
@@ -3858,9 +3964,8 @@
       <c r="T109" s="20"/>
       <c r="U109" s="20"/>
       <c r="V109" s="20"/>
-      <c r="W109" s="20"/>
-    </row>
-    <row r="110" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="110" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A110" s="20"/>
       <c r="B110" s="20"/>
       <c r="C110" s="20"/>
@@ -3883,9 +3988,8 @@
       <c r="T110" s="20"/>
       <c r="U110" s="20"/>
       <c r="V110" s="20"/>
-      <c r="W110" s="20"/>
-    </row>
-    <row r="111" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="111" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A111" s="20"/>
       <c r="B111" s="20"/>
       <c r="C111" s="20"/>
@@ -3908,9 +4012,8 @@
       <c r="T111" s="20"/>
       <c r="U111" s="20"/>
       <c r="V111" s="20"/>
-      <c r="W111" s="20"/>
-    </row>
-    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="112" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A112" s="20"/>
       <c r="B112" s="20"/>
       <c r="C112" s="20"/>
@@ -3933,9 +4036,8 @@
       <c r="T112" s="20"/>
       <c r="U112" s="20"/>
       <c r="V112" s="20"/>
-      <c r="W112" s="20"/>
-    </row>
-    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="113" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A113" s="20"/>
       <c r="B113" s="20"/>
       <c r="C113" s="20"/>
@@ -3958,9 +4060,8 @@
       <c r="T113" s="20"/>
       <c r="U113" s="20"/>
       <c r="V113" s="20"/>
-      <c r="W113" s="20"/>
-    </row>
-    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="114" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A114" s="20"/>
       <c r="B114" s="20"/>
       <c r="C114" s="20"/>
@@ -3983,9 +4084,8 @@
       <c r="T114" s="20"/>
       <c r="U114" s="20"/>
       <c r="V114" s="20"/>
-      <c r="W114" s="20"/>
-    </row>
-    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="115" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A115" s="20"/>
       <c r="B115" s="20"/>
       <c r="C115" s="20"/>
@@ -4008,9 +4108,8 @@
       <c r="T115" s="20"/>
       <c r="U115" s="20"/>
       <c r="V115" s="20"/>
-      <c r="W115" s="20"/>
-    </row>
-    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="116" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A116" s="20"/>
       <c r="B116" s="20"/>
       <c r="C116" s="20"/>
@@ -4033,9 +4132,8 @@
       <c r="T116" s="20"/>
       <c r="U116" s="20"/>
       <c r="V116" s="20"/>
-      <c r="W116" s="20"/>
-    </row>
-    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="117" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A117" s="20"/>
       <c r="B117" s="20"/>
       <c r="C117" s="20"/>
@@ -4058,7 +4156,6 @@
       <c r="T117" s="20"/>
       <c r="U117" s="20"/>
       <c r="V117" s="20"/>
-      <c r="W117" s="20"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -4075,9 +4172,16 @@
       <formula1>"Capital,Custeio"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="M2" r:id="rId1" xr:uid="{0C07EC8B-EB15-4D06-990F-242ABDE7980B}"/>
+    <hyperlink ref="M6" r:id="rId2" xr:uid="{0808E0BF-12C1-4966-ADF1-C00710038719}"/>
+    <hyperlink ref="M3" r:id="rId3" xr:uid="{B51B0197-E030-4AE1-A061-E3DD68EC318D}"/>
+    <hyperlink ref="M4" r:id="rId4" xr:uid="{FCCC70F8-4DE8-489C-91DD-73D0608B8252}"/>
+    <hyperlink ref="M5" r:id="rId5" xr:uid="{A0CAB60B-0939-475E-ABF3-AD1C0430748E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
pagina de orçamento botões
</commit_message>
<xml_diff>
--- a/banco_dados_orcamentario_onasp.xlsx
+++ b/banco_dados_orcamentario_onasp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://justicagovbr-my.sharepoint.com/personal/marcelo_cortez_mj_gov_br1/Documents/1. SENAPPEN/2. OUVIDORIA/GITHUB/FOMENTO-ONASP/FOMENTO-ONASP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{1210FA62-9861-4C19-87A7-EDB03CFB6BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4E6EC2F-A35C-40A2-A7C9-957E25A8392F}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{1210FA62-9861-4C19-87A7-EDB03CFB6BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50B4C5D1-A462-4AE6-93ED-ECD2D7EAE510}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="125">
   <si>
     <t>ID</t>
   </si>
@@ -387,6 +387,27 @@
   </si>
   <si>
     <t>https://sei.mj.gov.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=39457500&amp;id_documento=39457504</t>
+  </si>
+  <si>
+    <t>17/2025</t>
+  </si>
+  <si>
+    <t>https://sei.mj.gov.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=39355451&amp;id_documento=39355664</t>
+  </si>
+  <si>
+    <t>https://sei.mj.gov.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=39355451&amp;id_documento=39503055</t>
+  </si>
+  <si>
+    <t>19/2026</t>
+  </si>
+  <si>
+    <t>33/2026</t>
+  </si>
+  <si>
+    <t>https://sei.mj.gov.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=39355451&amp;id_documento=39630399</t>
+  </si>
+  <si>
+    <t>https://sei.mj.gov.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=39355451&amp;id_documento=39630647</t>
   </si>
 </sst>
 </file>
@@ -1081,18 +1102,42 @@
       <c r="O3" s="7">
         <v>46072</v>
       </c>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="7"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="7"/>
-      <c r="Y3" s="3"/>
-      <c r="Z3" s="4"/>
-      <c r="AA3" s="7"/>
+      <c r="P3" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q3" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="R3" s="7">
+        <v>46072</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="T3" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="U3" s="7">
+        <v>46084</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="W3" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="X3" s="7">
+        <v>46093</v>
+      </c>
+      <c r="Y3" s="3">
+        <v>34885945</v>
+      </c>
+      <c r="Z3" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="AA3" s="7">
+        <v>46093</v>
+      </c>
       <c r="AB3" s="3"/>
       <c r="AC3" s="4"/>
       <c r="AD3" s="7"/>
@@ -1178,18 +1223,42 @@
       <c r="O4" s="7">
         <v>46072</v>
       </c>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="7"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="7"/>
-      <c r="Y4" s="3"/>
-      <c r="Z4" s="4"/>
-      <c r="AA4" s="7"/>
+      <c r="P4" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q4" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="R4" s="7">
+        <v>46072</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="T4" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="U4" s="7">
+        <v>46084</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="W4" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="X4" s="7">
+        <v>46093</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>34885945</v>
+      </c>
+      <c r="Z4" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="AA4" s="7">
+        <v>46093</v>
+      </c>
       <c r="AB4" s="3"/>
       <c r="AC4" s="4"/>
       <c r="AD4" s="7"/>
@@ -1275,18 +1344,42 @@
       <c r="O5" s="7">
         <v>46072</v>
       </c>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="7"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="7"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="7"/>
-      <c r="Y5" s="3"/>
-      <c r="Z5" s="4"/>
-      <c r="AA5" s="7"/>
+      <c r="P5" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q5" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="R5" s="7">
+        <v>46072</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="T5" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="U5" s="7">
+        <v>46084</v>
+      </c>
+      <c r="V5" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="W5" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="X5" s="7">
+        <v>46093</v>
+      </c>
+      <c r="Y5" s="3">
+        <v>34885945</v>
+      </c>
+      <c r="Z5" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="AA5" s="7">
+        <v>46093</v>
+      </c>
       <c r="AB5" s="3"/>
       <c r="AC5" s="4"/>
       <c r="AD5" s="7"/>
@@ -1886,6 +1979,18 @@
   <hyperlinks>
     <hyperlink ref="Q2" r:id="rId1" xr:uid="{B25892D1-F18B-4FBE-AF84-DBCB517A9049}"/>
     <hyperlink ref="T2" r:id="rId2" xr:uid="{F0ECCEBE-E619-4578-B633-BD57600B82F4}"/>
+    <hyperlink ref="Q3" r:id="rId3" xr:uid="{D8511A91-9C29-4DD4-AD72-AF3C01C06693}"/>
+    <hyperlink ref="Q5" r:id="rId4" xr:uid="{DE5047F7-C413-4C53-B71A-1E7B46AB8F48}"/>
+    <hyperlink ref="Q4" r:id="rId5" xr:uid="{DB5CB5B2-185F-44CD-A786-F40E7D2A4F5F}"/>
+    <hyperlink ref="T5" r:id="rId6" xr:uid="{D784E0D7-3913-4094-A72D-B0A18EED820A}"/>
+    <hyperlink ref="T4" r:id="rId7" xr:uid="{8A175F20-F0B0-4968-BB19-531F316A94DC}"/>
+    <hyperlink ref="T3" r:id="rId8" xr:uid="{CB24C789-D60F-4EF6-9EE7-690C86DCE3B1}"/>
+    <hyperlink ref="W5" r:id="rId9" xr:uid="{9EE92907-6003-49E3-8194-AAD900A5851C}"/>
+    <hyperlink ref="W4" r:id="rId10" xr:uid="{C1F8C3B7-0736-4E91-BCF6-ED5FA4F394F6}"/>
+    <hyperlink ref="W3" r:id="rId11" xr:uid="{E9F1A9FA-45EA-41EB-A49B-1935826B59D7}"/>
+    <hyperlink ref="Z3" r:id="rId12" xr:uid="{AF09F900-A90A-47EF-934B-114C69291751}"/>
+    <hyperlink ref="Z4" r:id="rId13" xr:uid="{CA8A8774-3FC6-4C47-A620-67BEFFFE3214}"/>
+    <hyperlink ref="Z5" r:id="rId14" xr:uid="{09962DF5-4C88-4534-A301-58A456153B7D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>